<commit_message>
Swap two transposed unit prices and record the Rhodes quantities
The 2025 study priced the 50 kg wheeled CO2 refill at 2.90 EUR and the
6 kg ceiling unit at 31.46 EUR, which are transposed against their
neighbours (30 kg CO2 at 25.00, 12 kg ceiling at 4.00). Swapped on the
author's instruction, in the source data, both deliverables and the
application database.

This lowers the study rather than raising it: 4,781.16 EUR net and
5,928.64 EUR gross, against 5,999.47 EUR before, leaving 71.36 EUR of
headroom under the 6,000.00 EUR credit. No quantity reduction is needed.

Also records the study quantities as a draft request for the Rhodes
municipal unit for 2026 (unit_requests + 22 request_lines, 603 pieces),
so the figures live in the application alongside the catalogue.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018XBytJqxwkQKNMGqGDuTqk
</commit_message>
<xml_diff>
--- a/meletes/pyrosvestires-rodou-2026/ΠΥΡΟΣΒΕΣΤΗΡΕΣ_ΡΟΔΟΥ_2026.xlsx
+++ b/meletes/pyrosvestires-rodou-2026/ΠΥΡΟΣΒΕΣΤΗΡΕΣ_ΡΟΔΟΥ_2026.xlsx
@@ -2034,18 +2034,18 @@
         <v>44</v>
       </c>
       <c r="F18" s="9">
-        <v>2.9</v>
+        <v>31.46</v>
       </c>
       <c r="G18" s="10">
         <v>1</v>
       </c>
       <c r="H18" s="9">
         <f>IF(OR(F18="",G18=""),"",F18*G18)</f>
-        <v>2.9</v>
+        <v>31.46</v>
       </c>
       <c r="I18" s="9">
         <f>IF(F18="","",F18*(1+'ΣΗΜΕΙΩΣΕΙΣ'!$B$2))</f>
-        <v>3.596</v>
+        <v>39.010400000000004</v>
       </c>
       <c r="J18" s="11" t="s">
         <v>45</v>
@@ -2130,18 +2130,18 @@
         <v>50</v>
       </c>
       <c r="F21" s="9">
-        <v>31.46</v>
+        <v>2.9</v>
       </c>
       <c r="G21" s="10">
         <v>3</v>
       </c>
       <c r="H21" s="9">
         <f>IF(OR(F21="",G21=""),"",F21*G21)</f>
-        <v>94.38</v>
+        <v>8.7</v>
       </c>
       <c r="I21" s="9">
         <f>IF(F21="","",F21*(1+'ΣΗΜΕΙΩΣΕΙΣ'!$B$2))</f>
-        <v>39.010400000000004</v>
+        <v>3.596</v>
       </c>
       <c r="J21" s="11" t="s">
         <v>51</v>

</xml_diff>